<commit_message>
docs(register): OBS-E1 and OBS-E2 Fixed — 31 of 205, 20 of 46 Criticals
</commit_message>
<xml_diff>
--- a/doc/AUDIT_REGISTER_2026-08-04.xlsx
+++ b/doc/AUDIT_REGISTER_2026-08-04.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1556" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1558" uniqueCount="558">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -587,10 +587,16 @@
     <t xml:space="preserve">No centralised error tracking of any kind</t>
   </si>
   <si>
+    <t xml:space="preserve">shared/observability/error-reporter.js — every 5xx, uncaughtException and unhandledRejection reports with tenant/user/request_id/route/build. Dedupe + id normalisation + frame-drift stability + 20/min ceiling so the channel stays usable. 4xx and ZodError never reported. Commit e78a566.</t>
+  </si>
+  <si>
     <t xml:space="preserve">OBS-E2</t>
   </si>
   <si>
     <t xml:space="preserve">Frontend errors are completely invisible</t>
+  </si>
+  <si>
+    <t xml:space="preserve">POST /api/client-errors + client/src/lib/error-reporting.ts covering render, window 'error' and unhandledrejection. ErrorBoundary's dead onError hook now reports by default. sendBeacon survives the post-crash reload. Commit e78a566.</t>
   </si>
   <si>
     <t xml:space="preserve">OBS-L1</t>
@@ -3887,23 +3893,25 @@
       <c r="E63" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="F63" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G63" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H63" s="4"/>
+      <c r="F63" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G63" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H63" s="4" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>11</v>
@@ -3911,23 +3919,25 @@
       <c r="E64" s="4" t="s">
         <v>176</v>
       </c>
-      <c r="F64" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="H64" s="4"/>
+      <c r="F64" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G64" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>11</v>
@@ -3942,18 +3952,18 @@
         <v>14</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>11</v>
@@ -3971,13 +3981,13 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>11</v>
@@ -3992,18 +4002,18 @@
         <v>14</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B68" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>11</v>
@@ -4021,19 +4031,19 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="B69" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>27</v>
@@ -4045,19 +4055,19 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B70" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F70" s="4" t="s">
         <v>27</v>
@@ -4069,13 +4079,13 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>11</v>
@@ -4090,18 +4100,18 @@
         <v>14</v>
       </c>
       <c r="H71" s="4" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="B72" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D72" s="8" t="s">
         <v>25</v>
@@ -4116,18 +4126,18 @@
         <v>14</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B73" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D73" s="8" t="s">
         <v>25</v>
@@ -4145,19 +4155,19 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B74" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D74" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F74" s="4" t="s">
         <v>27</v>
@@ -4169,13 +4179,13 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B75" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D75" s="8" t="s">
         <v>25</v>
@@ -4190,18 +4200,18 @@
         <v>14</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B76" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D76" s="8" t="s">
         <v>25</v>
@@ -4216,24 +4226,24 @@
         <v>14</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B77" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D77" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F77" s="4" t="s">
         <v>27</v>
@@ -4245,13 +4255,13 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="B78" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D78" s="8" t="s">
         <v>25</v>
@@ -4269,13 +4279,13 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="B79" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D79" s="8" t="s">
         <v>25</v>
@@ -4290,18 +4300,18 @@
         <v>14</v>
       </c>
       <c r="H79" s="4" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="B80" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D80" s="8" t="s">
         <v>25</v>
@@ -4319,13 +4329,13 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B81" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D81" s="8" t="s">
         <v>25</v>
@@ -4343,13 +4353,13 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="B82" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D82" s="8" t="s">
         <v>25</v>
@@ -4364,24 +4374,24 @@
         <v>28</v>
       </c>
       <c r="H82" s="4" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B83" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D83" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>27</v>
@@ -4393,13 +4403,13 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B84" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D84" s="9" t="s">
         <v>44</v>
@@ -4417,13 +4427,13 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B85" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D85" s="9" t="s">
         <v>44</v>
@@ -4441,13 +4451,13 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="B86" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D86" s="9" t="s">
         <v>44</v>
@@ -4465,13 +4475,13 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B87" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D87" s="9" t="s">
         <v>44</v>
@@ -4489,13 +4499,13 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B88" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D88" s="9" t="s">
         <v>44</v>
@@ -4513,13 +4523,13 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B89" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D89" s="9" t="s">
         <v>44</v>
@@ -4534,24 +4544,24 @@
         <v>14</v>
       </c>
       <c r="H89" s="4" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>13</v>
@@ -4560,24 +4570,24 @@
         <v>14</v>
       </c>
       <c r="H90" s="4" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F91" s="6" t="s">
         <v>13</v>
@@ -4586,18 +4596,18 @@
         <v>14</v>
       </c>
       <c r="H91" s="4" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="B92" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>11</v>
@@ -4615,13 +4625,13 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B93" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>11</v>
@@ -4636,24 +4646,24 @@
         <v>14</v>
       </c>
       <c r="H93" s="4" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B94" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E94" s="4" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>27</v>
@@ -4665,19 +4675,19 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="B95" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D95" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E95" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F95" s="4" t="s">
         <v>27</v>
@@ -4689,13 +4699,13 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="B96" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D96" s="8" t="s">
         <v>25</v>
@@ -4713,13 +4723,13 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B97" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D97" s="8" t="s">
         <v>25</v>
@@ -4737,19 +4747,19 @@
     </row>
     <row r="98" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="B98" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="D98" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E98" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F98" s="6" t="s">
         <v>13</v>
@@ -4758,24 +4768,24 @@
         <v>14</v>
       </c>
       <c r="H98" s="4" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B99" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D99" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E99" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F99" s="4" t="s">
         <v>27</v>
@@ -4787,19 +4797,19 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="B100" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="D100" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E100" s="4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F100" s="4" t="s">
         <v>27</v>
@@ -4811,19 +4821,19 @@
     </row>
     <row r="101" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="B101" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D101" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E101" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F101" s="11" t="s">
         <v>130</v>
@@ -4832,24 +4842,24 @@
         <v>14</v>
       </c>
       <c r="H101" s="4" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B102" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="D102" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E102" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F102" s="4" t="s">
         <v>27</v>
@@ -4861,13 +4871,13 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="B103" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D103" s="9" t="s">
         <v>44</v>
@@ -4885,13 +4895,13 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="B104" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D104" s="9" t="s">
         <v>44</v>
@@ -4909,19 +4919,19 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="3" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="B105" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D105" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E105" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F105" s="4" t="s">
         <v>27</v>
@@ -4933,19 +4943,19 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="B106" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D106" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E106" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F106" s="4" t="s">
         <v>27</v>
@@ -4957,19 +4967,19 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="3" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B107" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D107" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E107" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F107" s="4" t="s">
         <v>27</v>
@@ -4981,19 +4991,19 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="B108" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D108" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E108" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F108" s="4" t="s">
         <v>27</v>
@@ -5005,19 +5015,19 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="3" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B109" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D109" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E109" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F109" s="4" t="s">
         <v>27</v>
@@ -5029,19 +5039,19 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B110" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D110" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E110" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F110" s="4" t="s">
         <v>27</v>
@@ -5053,13 +5063,13 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="3" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="B111" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D111" s="9" t="s">
         <v>44</v>
@@ -5077,19 +5087,19 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="B112" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D112" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E112" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F112" s="4" t="s">
         <v>27</v>
@@ -5101,19 +5111,19 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="3" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="B113" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="D113" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E113" s="4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F113" s="4" t="s">
         <v>27</v>
@@ -5125,19 +5135,19 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="B114" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D114" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E114" s="4" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F114" s="4" t="s">
         <v>27</v>
@@ -5149,19 +5159,19 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="3" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B115" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="D115" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E115" s="4" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="F115" s="4" t="s">
         <v>27</v>
@@ -5173,19 +5183,19 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="B116" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E116" s="4" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="F116" s="4" t="s">
         <v>27</v>
@@ -5197,19 +5207,19 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="3" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B117" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D117" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E117" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>27</v>
@@ -5221,19 +5231,19 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B118" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="D118" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E118" s="4" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="F118" s="4" t="s">
         <v>27</v>
@@ -5245,22 +5255,22 @@
     </row>
     <row r="119" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="3" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="B119" s="4" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="D119" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E119" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F119" s="12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G119" s="4" t="s">
         <v>28</v>
@@ -5269,13 +5279,13 @@
     </row>
     <row r="120" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="B120" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>11</v>
@@ -5290,18 +5300,18 @@
         <v>14</v>
       </c>
       <c r="H120" s="4" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="3" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B121" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>11</v>
@@ -5319,13 +5329,13 @@
     </row>
     <row r="122" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="B122" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>11</v>
@@ -5340,24 +5350,24 @@
         <v>14</v>
       </c>
       <c r="H122" s="4" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="3" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="B123" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="D123" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E123" s="4" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="F123" s="4" t="s">
         <v>27</v>
@@ -5369,13 +5379,13 @@
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B124" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="D124" s="8" t="s">
         <v>25</v>
@@ -5393,13 +5403,13 @@
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="3" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="B125" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="D125" s="8" t="s">
         <v>25</v>
@@ -5417,13 +5427,13 @@
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="B126" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="D126" s="8" t="s">
         <v>25</v>
@@ -5441,13 +5451,13 @@
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="3" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B127" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D127" s="8" t="s">
         <v>25</v>
@@ -5465,13 +5475,13 @@
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="B128" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="D128" s="8" t="s">
         <v>25</v>
@@ -5489,13 +5499,13 @@
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="3" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B129" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="D129" s="8" t="s">
         <v>25</v>
@@ -5513,13 +5523,13 @@
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="B130" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="D130" s="8" t="s">
         <v>25</v>
@@ -5537,13 +5547,13 @@
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="3" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="B131" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D131" s="8" t="s">
         <v>25</v>
@@ -5561,13 +5571,13 @@
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="B132" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="D132" s="9" t="s">
         <v>44</v>
@@ -5585,13 +5595,13 @@
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="3" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="B133" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="D133" s="9" t="s">
         <v>44</v>
@@ -5609,13 +5619,13 @@
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="B134" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="D134" s="9" t="s">
         <v>44</v>
@@ -5633,13 +5643,13 @@
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="3" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="B135" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="D135" s="9" t="s">
         <v>44</v>
@@ -5657,19 +5667,19 @@
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="B136" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C136" s="4" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="D136" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E136" s="4" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="F136" s="4" t="s">
         <v>27</v>
@@ -5681,13 +5691,13 @@
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="3" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="B137" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C137" s="4" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="D137" s="9" t="s">
         <v>44</v>
@@ -5705,13 +5715,13 @@
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="B138" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C138" s="4" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="D138" s="10" t="s">
         <v>69</v>
@@ -5729,13 +5739,13 @@
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="3" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B139" s="4" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="C139" s="4" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D139" s="10" t="s">
         <v>69</v>
@@ -5753,19 +5763,19 @@
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="B140" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C140" s="4" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="D140" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E140" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F140" s="4" t="s">
         <v>27</v>
@@ -5777,19 +5787,19 @@
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="B141" s="4" t="s">
         <v>373</v>
       </c>
-      <c r="B141" s="4" t="s">
-        <v>371</v>
-      </c>
       <c r="C141" s="4" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="D141" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E141" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F141" s="4" t="s">
         <v>27</v>
@@ -5801,19 +5811,19 @@
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="B142" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C142" s="4" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D142" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E142" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F142" s="4" t="s">
         <v>27</v>
@@ -5825,19 +5835,19 @@
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="3" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="B143" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C143" s="4" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="D143" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E143" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F143" s="4" t="s">
         <v>27</v>
@@ -5849,19 +5859,19 @@
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="B144" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C144" s="4" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="D144" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E144" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F144" s="6" t="s">
         <v>13</v>
@@ -5870,24 +5880,24 @@
         <v>14</v>
       </c>
       <c r="H144" s="4" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="3" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B145" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C145" s="4" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="D145" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E145" s="4" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F145" s="6" t="s">
         <v>13</v>
@@ -5896,24 +5906,24 @@
         <v>14</v>
       </c>
       <c r="H145" s="4" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="B146" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C146" s="4" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="D146" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E146" s="4" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F146" s="4" t="s">
         <v>27</v>
@@ -5925,19 +5935,19 @@
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="3" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B147" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C147" s="4" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="D147" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E147" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F147" s="4" t="s">
         <v>27</v>
@@ -5949,19 +5959,19 @@
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="B148" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C148" s="4" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="D148" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E148" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F148" s="4" t="s">
         <v>27</v>
@@ -5973,19 +5983,19 @@
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="3" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="B149" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C149" s="4" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="D149" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E149" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F149" s="4" t="s">
         <v>27</v>
@@ -5997,19 +6007,19 @@
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B150" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C150" s="4" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="D150" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E150" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F150" s="4" t="s">
         <v>27</v>
@@ -6021,19 +6031,19 @@
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="3" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="B151" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C151" s="4" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="D151" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E151" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F151" s="4" t="s">
         <v>27</v>
@@ -6045,19 +6055,19 @@
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B152" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C152" s="4" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="D152" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E152" s="4" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F152" s="4" t="s">
         <v>27</v>
@@ -6069,19 +6079,19 @@
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="3" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="B153" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C153" s="4" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="D153" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E153" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F153" s="4" t="s">
         <v>27</v>
@@ -6093,19 +6103,19 @@
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B154" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C154" s="4" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="D154" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E154" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F154" s="4" t="s">
         <v>27</v>
@@ -6117,19 +6127,19 @@
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="3" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="B155" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C155" s="4" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="D155" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E155" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F155" s="4" t="s">
         <v>27</v>
@@ -6141,19 +6151,19 @@
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="B156" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C156" s="4" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="D156" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E156" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F156" s="4" t="s">
         <v>27</v>
@@ -6165,19 +6175,19 @@
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="3" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="B157" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C157" s="4" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="D157" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E157" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F157" s="4" t="s">
         <v>27</v>
@@ -6189,19 +6199,19 @@
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="B158" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C158" s="4" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="D158" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E158" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F158" s="4" t="s">
         <v>27</v>
@@ -6213,19 +6223,19 @@
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="3" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B159" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C159" s="4" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="D159" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E159" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F159" s="4" t="s">
         <v>27</v>
@@ -6237,19 +6247,19 @@
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="B160" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C160" s="4" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="D160" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E160" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F160" s="6" t="s">
         <v>13</v>
@@ -6258,24 +6268,24 @@
         <v>14</v>
       </c>
       <c r="H160" s="4" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="3" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B161" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C161" s="4" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="D161" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E161" s="4" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="F161" s="4" t="s">
         <v>27</v>
@@ -6287,19 +6297,19 @@
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="B162" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C162" s="4" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="D162" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E162" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F162" s="4" t="s">
         <v>27</v>
@@ -6311,19 +6321,19 @@
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="3" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="B163" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C163" s="4" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="D163" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E163" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F163" s="4" t="s">
         <v>27</v>
@@ -6335,19 +6345,19 @@
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="B164" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C164" s="4" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="D164" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E164" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F164" s="6" t="s">
         <v>13</v>
@@ -6356,24 +6366,24 @@
         <v>14</v>
       </c>
       <c r="H164" s="4" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="3" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="B165" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C165" s="4" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="D165" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E165" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F165" s="4" t="s">
         <v>27</v>
@@ -6385,45 +6395,45 @@
     </row>
     <row r="166" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="B166" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C166" s="4" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="D166" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E166" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F166" s="11" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="G166" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H166" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="3" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B167" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C167" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="D167" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E167" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F167" s="4" t="s">
         <v>27</v>
@@ -6435,19 +6445,19 @@
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="B168" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C168" s="4" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="D168" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E168" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F168" s="4" t="s">
         <v>27</v>
@@ -6459,19 +6469,19 @@
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="3" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B169" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C169" s="4" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="D169" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E169" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F169" s="4" t="s">
         <v>27</v>
@@ -6483,19 +6493,19 @@
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B170" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C170" s="4" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="D170" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E170" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F170" s="4" t="s">
         <v>27</v>
@@ -6507,19 +6517,19 @@
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="3" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="B171" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C171" s="4" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="D171" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E171" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F171" s="6" t="s">
         <v>13</v>
@@ -6528,24 +6538,24 @@
         <v>14</v>
       </c>
       <c r="H171" s="4" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="B172" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C172" s="4" t="s">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="D172" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E172" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F172" s="4" t="s">
         <v>27</v>
@@ -6557,19 +6567,19 @@
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="3" t="s">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="B173" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C173" s="4" t="s">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="D173" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E173" s="4" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="F173" s="4" t="s">
         <v>27</v>
@@ -6581,19 +6591,19 @@
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B174" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C174" s="4" t="s">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="D174" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E174" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F174" s="4" t="s">
         <v>27</v>
@@ -6605,19 +6615,19 @@
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="3" t="s">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B175" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C175" s="4" t="s">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="D175" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E175" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F175" s="4" t="s">
         <v>27</v>
@@ -6629,19 +6639,19 @@
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="B176" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C176" s="4" t="s">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="D176" s="13" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E176" s="4" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="F176" s="4" t="s">
         <v>27</v>
@@ -6653,19 +6663,19 @@
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="3" t="s">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B177" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C177" s="4" t="s">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="D177" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E177" s="4" t="s">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="F177" s="6" t="s">
         <v>13</v>
@@ -6674,24 +6684,24 @@
         <v>14</v>
       </c>
       <c r="H177" s="4" t="s">
-        <v>459</v>
+        <v>461</v>
       </c>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="B178" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C178" s="4" t="s">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="D178" s="13" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E178" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F178" s="4" t="s">
         <v>27</v>
@@ -6703,19 +6713,19 @@
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="3" t="s">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="B179" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C179" s="4" t="s">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="D179" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E179" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F179" s="4" t="s">
         <v>27</v>
@@ -6727,19 +6737,19 @@
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="B180" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C180" s="4" t="s">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="D180" s="14" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E180" s="4" t="s">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="F180" s="4" t="s">
         <v>27</v>
@@ -6751,19 +6761,19 @@
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="3" t="s">
+        <v>470</v>
+      </c>
+      <c r="B181" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="C181" s="4" t="s">
+        <v>471</v>
+      </c>
+      <c r="D181" s="14" t="s">
         <v>468</v>
       </c>
-      <c r="B181" s="4" t="s">
-        <v>371</v>
-      </c>
-      <c r="C181" s="4" t="s">
-        <v>469</v>
-      </c>
-      <c r="D181" s="14" t="s">
-        <v>466</v>
-      </c>
       <c r="E181" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F181" s="4" t="s">
         <v>27</v>
@@ -6775,19 +6785,19 @@
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A182" s="3" t="s">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="B182" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C182" s="4" t="s">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="D182" s="14" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="E182" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F182" s="4" t="s">
         <v>27</v>
@@ -6799,19 +6809,19 @@
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A183" s="3" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="B183" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C183" s="4" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="D183" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E183" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F183" s="4" t="s">
         <v>27</v>
@@ -6823,19 +6833,19 @@
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A184" s="3" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="B184" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C184" s="4" t="s">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="D184" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E184" s="4" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="F184" s="4" t="s">
         <v>27</v>
@@ -6847,22 +6857,22 @@
     </row>
     <row r="185" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A185" s="3" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B185" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C185" s="4" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="D185" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E185" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F185" s="12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G185" s="4" t="s">
         <v>28</v>
@@ -6871,22 +6881,22 @@
     </row>
     <row r="186" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A186" s="3" t="s">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="B186" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C186" s="4" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="D186" s="10" t="s">
         <v>69</v>
       </c>
       <c r="E186" s="4" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F186" s="12" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="G186" s="4" t="s">
         <v>28</v>
@@ -6895,13 +6905,13 @@
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A187" s="3" t="s">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="B187" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C187" s="4" t="s">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="D187" s="5" t="s">
         <v>11</v>
@@ -6919,13 +6929,13 @@
     </row>
     <row r="188" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A188" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="B188" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="B188" s="4" t="s">
-        <v>481</v>
-      </c>
       <c r="C188" s="4" t="s">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="D188" s="5" t="s">
         <v>11</v>
@@ -6940,24 +6950,24 @@
         <v>14</v>
       </c>
       <c r="H188" s="4" t="s">
-        <v>485</v>
+        <v>487</v>
       </c>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A189" s="3" t="s">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="B189" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C189" s="4" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="D189" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E189" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F189" s="11" t="s">
         <v>130</v>
@@ -6966,24 +6976,24 @@
         <v>14</v>
       </c>
       <c r="H189" s="4" t="s">
-        <v>489</v>
+        <v>491</v>
       </c>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A190" s="3" t="s">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="B190" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C190" s="4" t="s">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="D190" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E190" s="4" t="s">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="F190" s="4" t="s">
         <v>27</v>
@@ -6995,13 +7005,13 @@
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A191" s="3" t="s">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B191" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C191" s="4" t="s">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="D191" s="5" t="s">
         <v>11</v>
@@ -7019,45 +7029,45 @@
     </row>
     <row r="192" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A192" s="3" t="s">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="B192" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C192" s="4" t="s">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="D192" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E192" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F192" s="6" t="s">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="G192" s="7" t="s">
         <v>14</v>
       </c>
       <c r="H192" s="4" t="s">
-        <v>498</v>
+        <v>500</v>
       </c>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A193" s="3" t="s">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="B193" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C193" s="4" t="s">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="D193" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E193" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F193" s="4" t="s">
         <v>27</v>
@@ -7069,13 +7079,13 @@
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A194" s="3" t="s">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="B194" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C194" s="4" t="s">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="D194" s="8" t="s">
         <v>25</v>
@@ -7093,19 +7103,19 @@
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A195" s="3" t="s">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="B195" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C195" s="4" t="s">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="D195" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E195" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F195" s="4" t="s">
         <v>27</v>
@@ -7117,13 +7127,13 @@
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A196" s="3" t="s">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="B196" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C196" s="4" t="s">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="D196" s="8" t="s">
         <v>25</v>
@@ -7141,19 +7151,19 @@
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A197" s="3" t="s">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="B197" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C197" s="4" t="s">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="D197" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E197" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F197" s="4" t="s">
         <v>27</v>
@@ -7165,13 +7175,13 @@
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A198" s="3" t="s">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="B198" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C198" s="4" t="s">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="D198" s="8" t="s">
         <v>25</v>
@@ -7189,13 +7199,13 @@
     </row>
     <row r="199" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A199" s="3" t="s">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="B199" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C199" s="4" t="s">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="D199" s="9" t="s">
         <v>44</v>
@@ -7210,24 +7220,24 @@
         <v>14</v>
       </c>
       <c r="H199" s="4" t="s">
-        <v>513</v>
+        <v>515</v>
       </c>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A200" s="3" t="s">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B200" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C200" s="4" t="s">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="D200" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E200" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F200" s="4" t="s">
         <v>27</v>
@@ -7239,19 +7249,19 @@
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A201" s="3" t="s">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B201" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C201" s="4" t="s">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="D201" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E201" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F201" s="4" t="s">
         <v>27</v>
@@ -7263,19 +7273,19 @@
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A202" s="3" t="s">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="B202" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C202" s="4" t="s">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="D202" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E202" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F202" s="4" t="s">
         <v>27</v>
@@ -7287,13 +7297,13 @@
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A203" s="3" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="B203" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C203" s="4" t="s">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="D203" s="9" t="s">
         <v>44</v>
@@ -7311,19 +7321,19 @@
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A204" s="3" t="s">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="B204" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C204" s="4" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="D204" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E204" s="4" t="s">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="F204" s="4" t="s">
         <v>27</v>
@@ -7335,13 +7345,13 @@
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A205" s="3" t="s">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="B205" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C205" s="4" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="D205" s="9" t="s">
         <v>44</v>
@@ -7359,19 +7369,19 @@
     </row>
     <row r="206" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A206" s="3" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="B206" s="4" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="C206" s="4" t="s">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="D206" s="9" t="s">
         <v>44</v>
       </c>
       <c r="E206" s="4" t="s">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="F206" s="4" t="s">
         <v>27</v>
@@ -7381,21 +7391,21 @@
       </c>
       <c r="H206" s="4"/>
     </row>
-    <row r="207" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="207" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A207" s="3" t="s">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B207" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C207" s="4" t="s">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="D207" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E207" s="4" t="s">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="F207" s="6" t="s">
         <v>13</v>
@@ -7404,24 +7414,24 @@
         <v>14</v>
       </c>
       <c r="H207" s="4" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="208" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="208" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A208" s="3" t="s">
-        <v>533</v>
+        <v>535</v>
       </c>
       <c r="B208" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C208" s="4" t="s">
-        <v>534</v>
+        <v>536</v>
       </c>
       <c r="D208" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E208" s="4" t="s">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="F208" s="6" t="s">
         <v>13</v>
@@ -7430,18 +7440,18 @@
         <v>14</v>
       </c>
       <c r="H208" s="4" t="s">
-        <v>536</v>
-      </c>
-    </row>
-    <row r="209" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="209" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A209" s="3" t="s">
-        <v>537</v>
+        <v>539</v>
       </c>
       <c r="B209" s="4" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C209" s="4" t="s">
-        <v>538</v>
+        <v>540</v>
       </c>
       <c r="D209" s="5" t="s">
         <v>11</v>
@@ -7456,18 +7466,18 @@
         <v>14</v>
       </c>
       <c r="H209" s="4" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="210" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="210" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A210" s="3" t="s">
-        <v>540</v>
+        <v>542</v>
       </c>
       <c r="B210" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C210" s="4" t="s">
-        <v>541</v>
+        <v>543</v>
       </c>
       <c r="D210" s="8" t="s">
         <v>25</v>
@@ -7482,24 +7492,24 @@
         <v>14</v>
       </c>
       <c r="H210" s="4" t="s">
-        <v>542</v>
-      </c>
-    </row>
-    <row r="211" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="211" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A211" s="3" t="s">
-        <v>543</v>
+        <v>545</v>
       </c>
       <c r="B211" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C211" s="4" t="s">
-        <v>544</v>
+        <v>546</v>
       </c>
       <c r="D211" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E211" s="4" t="s">
-        <v>545</v>
+        <v>547</v>
       </c>
       <c r="F211" s="4" t="s">
         <v>27</v>
@@ -7508,18 +7518,18 @@
         <v>14</v>
       </c>
       <c r="H211" s="4" t="s">
-        <v>546</v>
-      </c>
-    </row>
-    <row r="212" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="212" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A212" s="3" t="s">
-        <v>547</v>
+        <v>549</v>
       </c>
       <c r="B212" s="4" t="s">
         <v>174</v>
       </c>
       <c r="C212" s="4" t="s">
-        <v>548</v>
+        <v>550</v>
       </c>
       <c r="D212" s="10" t="s">
         <v>69</v>
@@ -7534,7 +7544,7 @@
         <v>14</v>
       </c>
       <c r="H212" s="4" t="s">
-        <v>549</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -7570,7 +7580,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>550</v>
+        <v>552</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -7582,7 +7592,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>551</v>
+        <v>553</v>
       </c>
       <c r="B2" s="16"/>
       <c r="C2" s="16"/>
@@ -7613,19 +7623,19 @@
         <v>25</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="E4" s="20" t="s">
         <v>44</v>
       </c>
       <c r="F4" s="20" t="s">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="G4" s="20" t="s">
         <v>69</v>
       </c>
       <c r="H4" s="20" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7729,7 +7739,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="21" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B8" s="22" t="n">
         <f aca="false">COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,B$4)</f>
@@ -7762,7 +7772,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="B9" s="22" t="n">
         <f aca="false">COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,B$4)</f>
@@ -7795,7 +7805,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="B10" s="22" t="n">
         <f aca="false">COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,B$4)</f>
@@ -7828,7 +7838,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="21" t="s">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="B11" s="22" t="n">
         <f aca="false">COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,B$4)</f>
@@ -7861,7 +7871,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="21" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="B12" s="23" t="n">
         <f aca="false">SUM(B5:B11)</f>
@@ -7904,7 +7914,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>553</v>
+        <v>555</v>
       </c>
       <c r="B14" s="22"/>
       <c r="C14" s="22"/>
@@ -7920,7 +7930,7 @@
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">COUNTIF(Register!$F$2:$F$206,$A15)</f>
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C15" s="22"/>
       <c r="D15" s="22"/>
@@ -7950,7 +7960,7 @@
       </c>
       <c r="B17" s="22" t="n">
         <f aca="false">COUNTIF(Register!$F$2:$F$206,"Fixed")</f>
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C17" s="22"/>
       <c r="D17" s="22"/>
@@ -7961,7 +7971,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>554</v>
+        <v>556</v>
       </c>
       <c r="B18" s="22" t="n">
         <f aca="false">COUNTIF(Register!$F$2:$F$206,$A18)</f>
@@ -7976,7 +7986,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="21" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="B19" s="22" t="n">
         <f aca="false">COUNTIF(Register!$F$2:$F$206,$A19)</f>
@@ -7991,11 +8001,11 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>555</v>
+        <v>557</v>
       </c>
       <c r="B20" s="22" t="n">
         <f aca="false">COUNTIF(Register!$G$2:$G$206,"Verified in code")</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C20" s="22"/>
       <c r="D20" s="22"/>

</xml_diff>

<commit_message>
Refactor tenant registry tests and add comprehensive WMS inventory tests
- Renamed `FakePool` to `mockFakePool` in tenant registry tests for clarity.
- Introduced a new test file `wms-inventory.test.js` to cover WMS inventory functionality.
- Implemented a mock in-memory Postgres database for testing inventory operations.
- Added tests to validate inventory movement, concurrency handling, and state transitions.
- Ensured that inventory operations respect negative stock constraints and transaction integrity.
</commit_message>
<xml_diff>
--- a/doc/AUDIT_REGISTER_2026-08-04.xlsx
+++ b/doc/AUDIT_REGISTER_2026-08-04.xlsx
@@ -188,7 +188,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -330,6 +330,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2202,15 +2205,19 @@
       </c>
       <c r="F37" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G37" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H37" s="48" t="inlineStr">
+        <is>
+          <t>~60 tenant columns are REFERENCES app_user(user_id); identity is pinned to the LIVE schema while business writes go to whichever schema the request selected, so a valid live user id raises 23503 beside sandbox data. emit.js guarded its own actor columns; the finding was that the guard was applied INCONSISTENTLY. All 15 raw `&lt;x&gt;_by: actor.user_id` writes across 13 services now go through resolveActorId (governance, extra_charge_simulation, margin_simulation, credit_note, final_invoice, journal_entry, appraisal, hr_query, hr_sanction, success_story, smartcomm, report, inventory.moved_by, cycle_count.counted_by). PREVENTION, because this is a class of defect that repairs itself back into existence the next time somebody adds an `_by` column: scripts/check-actor-fk-guard.js fails the build on a raw one with the reason and the remedy, wired into ci.yaml. Verified to bite (reintroducing one fails it) and green after. wms-inventory.test.js now models app_user per-schema and asserts both directions — the actor resolves when present, and a NULL is written rather than the movement failing when absent.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="25">
       <c r="A38" s="27" t="inlineStr">
@@ -2282,15 +2289,19 @@
       </c>
       <c r="F39" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G39" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H39" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H39" s="28" t="inlineStr">
+        <is>
+          <t>migrateAllTenants was a bare loop with no try/catch, so the first failure aborted it and split the fleet at an arbitrary point with NOTHING RECORDING WHERE — during a deploy, while the new image expecting the new schema rolled out to all of them. It now continues past a failure, records per-tenant outcome, and throws afterwards so the deploy still goes red having done as much as it safely could. Continue rather than stop deliberately: a tenant-specific cause should not punish everyone after it in the list, and a systematic cause produces 'all 12 failed' rather than 'the first one failed'. Plus fleetSchemaStatus() + scripts/db/fleet-status.js, reading each tenant's own ledger so it reports what was APPLIED not what someone believes was; wired into CI.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="25">
       <c r="A40" s="27" t="inlineStr">
@@ -2320,15 +2331,19 @@
       </c>
       <c r="F40" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G40" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H40" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H40" s="28" t="inlineStr">
+        <is>
+          <t>Migration 0503 adds the missing created_at with ADD COLUMN IF NOT EXISTS — the right instrument because the two CREATE TABLE files disagree about history and this converges both without needing to know which ran. The column is documented as 'not before this migration' rather than pretending its backfilled now() is authoritative for historical rows. Neither original file is edited: editing an applied migration changes nothing on a database that already ran it. Plus scripts/db/check-schema-drift.js in CI. Its first version compared table names GLOBALLY and reported 4 conflicts, 3 of them false — tenant and platform are separate databases that legitimately share ai_vendor_credential, ai_document and ai_chunk. Scoped per database it reports exactly the one real conflict, and it recognises a later ALTER as the resolution so it does not stay red forever after the fix. Proven both ways: red with 0503 reverted, green with it restored.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="25">
       <c r="A41" s="27" t="inlineStr">
@@ -2736,15 +2751,19 @@
       </c>
       <c r="F50" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G50" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H50" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H50" s="48" t="inlineStr">
+        <is>
+          <t>migrations/tenant/0505, part 2. A DECISION, recorded rather than a behaviour change: ON UPDATE stays NO ACTION on the natural text keys (chart_of_accounts.code, currency.code). The audit's own reading is that this is arguably CORRECT for a statutory chart — a posted OHADA code identifies those postings forever, and ON UPDATE CASCADE would make a rename succeed silently across twelve tables, rewriting the meaning of historical entries with no audit record that the account was ever called anything else. The complaint was that it was undocumented while the COA service exposes edit paths, so a maintainer could not tell a deliberate restriction from an oversight and the next person to hit the FK violation would quite likely 'fix' it with CASCADE. Now a COMMENT ON COLUMN on both, which lives in the database, survives dump/restore, and shows up in \d+.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="25">
       <c r="A51" s="27" t="inlineStr">
@@ -2812,15 +2831,19 @@
       </c>
       <c r="F52" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G52" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H52" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H52" s="48" t="inlineStr">
+        <is>
+          <t>migrations/tenant/0506_leave_approval_repair.sql. 0467/0468 end their DO blocks with EXCEPTION WHEN OTHERS THEN NULL, so any failure was discarded and the migration recorded SUCCESS — leaving the tenant with no leave-approval workflow, which makes executor.start() return autoApproved, the calling module discard that flag, and the request sit forever without being rejected or queued (W8/W11). Not editable in place: the migrator keys the ledger on filename (DATA 3.1) and both are applied everywhere, so only a new file reaches an affected tenant — the same reasoning 0492 gives for the identical defect in 0469. Takes 0492's treatment: idempotent (no-op where 0467/0468 worked), narrow exception scope, and RAISE WARNING naming the schema, the SQLSTATE and the consequence instead of silence. Still non-fatal — a convenience seed must not block a deploy — but never again invisible. Reports how many missing approval tasks it opened.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="15" customHeight="1" s="25">
       <c r="A53" s="27" t="inlineStr">
@@ -2934,15 +2957,19 @@
       </c>
       <c r="F55" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G55" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H55" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H55" s="48" t="inlineStr">
+        <is>
+          <t>provisionTenant's five platform writes (tenant upsert, tenant_database, subdomain, status='LIVE', audit) ran on a bare client with no BEGIN, each autocommitting, so a failure part-way left a tenant registered with no database row or no subdomain, or stuck in PROVISIONING with its schema fully built and nothing routing to it — every one needing a human to unpick. Now one transaction with ROLLBACK on failure (and a failed ROLLBACK never masks the original error). The tenant DATABASE stays deliberately outside it and the code says why: CREATE DATABASE cannot participate in a transaction on another connection, and the asymmetry is the right way round — an orphaned database with no platform row is inert and re-provisioning is idempotent, whereas a platform row pointing at a database that does not exist routes live traffic into a 500. wipeSandbox likewise: DROP SCHEMA -&gt; CREATE -&gt; ledger DELETE -&gt; re-apply -&gt; mirror is now atomic, and Postgres CAN roll those back, so a crash mid-rebuild no longer leaves a tenant with NO sandbox schema and a ledger claiming the scopes were applied (which made self-healing impossible). Verified by the tenant-provisioning tests, including the tripwire this batch deliberately left behind: the test that asserted the OLD non-transactional behaviour failed on the fix and was rewritten to assert the new one, plus rollback and no-re-projection cases.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="25">
       <c r="A56" s="27" t="inlineStr">
@@ -3014,15 +3041,19 @@
       </c>
       <c r="F57" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G57" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H57" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H57" s="48" t="inlineStr">
+        <is>
+          <t>migrations/tenant/0504, part 1. Seven composite indexes on columns that gate correctness-critical queries: invoice(status,type), payment_allocation(invoice_id), journal_line(account_code,entry_id), journal_entry(entity_id,period_id,status), stock_movement(inventory_item_id,moved_at DESC), depreciation_schedule(asset_id,posted), and accounting_period(entity_id,starts_on,ends_on) — that last backs getPeriodForDate, which runs on EVERY journal post and had no supporting index at all. Plain CREATE INDEX IF NOT EXISTS, not CONCURRENTLY, for the reason 0496/0500 already document (the migrator sends each file as one multi-statement simple query, which Postgres wraps in an implicit transaction where CONCURRENTLY cannot run). Rollback stated in the header. VERIFIED BY PARSING ONLY — see the note on 0505.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="25">
       <c r="A58" s="27" t="inlineStr">
@@ -3052,15 +3083,19 @@
       </c>
       <c r="F58" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G58" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H58" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H58" s="48" t="inlineStr">
+        <is>
+          <t>migrations/tenant/0505, part 1. The KB §23.14 invariant ('a dictionary item cannot exist without at least one complete posting rule') was enforced by a constraint trigger AFTER INSERT ON dictionary_item only — it stopped you creating a rule-less item and did nothing about deleting the last rule out from under one that already existed. Consequence is not cosmetic: an item with no posting rule has no account to post to, so a costing line referencing it fails at posting time, long after the delete, in a different module, with an error naming neither. Closed from the other side with a DEFERRABLE constraint trigger AFTER DELETE OR UPDATE on posting_rule. DEFERRABLE matching 0200, so a legitimate replace-all-rules transaction still works — the check runs at COMMIT. AFTER UPDATE too, because re-pointing a rule's dictionary_item_id orphans the old item just as surely as deleting it. Skips the check when the item itself is gone, since deleting an item with its rules is legitimate.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="25">
       <c r="A59" s="27" t="inlineStr">
@@ -3888,15 +3923,19 @@
       </c>
       <c r="F78" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G78" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H78" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H78" s="28" t="inlineStr">
+        <is>
+          <t>New shared/observability/business-metrics.js: six probes over data that already existed — invoices posted by status, journal entries, approvals pending bucketed by age, undelivered/DEAD orchestration events, ledger writes per hour, and depreciation rows posted with no entry (the one that would have caught DATA 5.5, where uptime was 100%, error rate zero, and the only symptom was a number that should have been rising and was flat). Required adding GAUGE support to metrics.js, which had counters and histograms only — modelling a level as a counter makes rate() meaningless and a decrease read as a process restart. Refreshes on a timer rather than per scrape, because a 15s poll across the fleet is its own load problem against the PERF S1 connection budget. A failing tenant is reported AS a metric (collect_ok 0) rather than breaking the endpoint — proven with an unreachable tenant in the fleet, and with a probe whose table does not exist being skipped at debug.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="15" customHeight="1" s="25">
       <c r="A79" s="27" t="inlineStr">
@@ -4170,15 +4209,19 @@
       </c>
       <c r="F85" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G85" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H85" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H85" s="48" t="inlineStr">
+        <is>
+          <t>Two changes. (1) LEVEL: the eight paths the audit names as REAL swallowed failures move warn -&gt; error — costing-approval draft-invoice sync, email and push delivery (x2 each), approval notifications (x2), and AI usage/spend logging — so an alert keyed on level&gt;=error now sees them. Deliberately NOT a blanket conversion: a cache miss or a geocode timeout is a genuine degrade, and promoting those would drown the eight that matter. (2) STACKS: `{ err: err.message }` discards the stack, which was the other half of the finding. All 74 call sites across 49 files now pass the Error object, so pino's default err serializer keeps type, message and stack. Applied only inside logger.* calls — `err: err.message` feeding a jsonb column or an error-report payload is left alone, because an Error there serialises to '{}' and converting would LOSE the message rather than gain a stack. REDACT_PATHS already censors err.detail, so the pg-error leak stays closed.</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="25">
       <c r="A86" s="27" t="inlineStr">
@@ -4754,15 +4797,19 @@
       </c>
       <c r="F99" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G99" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H99" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H99" s="48" t="inlineStr">
+        <is>
+          <t>Lifecycle transitions were gated four different ways. All twelve flat-gated modules now use the shared requireTransitionPermission with a declared TRANSITION_ACTION map, validator FIRST so the target state is checked against the enum before it selects its own gate. The split follows the design the helper already documents: ADVANCING a record is `edit`; a decision that ends it, or that is irreversible outside the system (DISPATCHED, SIGNED, CLOSED, DONE, CANCELLED), is `approve`. Unlisted states fall back to `approve` — fails closed. purchase_request.routes.js's local reimplementation of the helper is deleted in favour of the shared import. One deliberate LOOSENING, flagged: proposal was flat `approve` for every target, so only approvers could SUBMIT — the exact bug PERMISSION_SWEEP_BACKLOG §A and the helper's own header describe. DRAFT/IN_REVIEW/SENT relax to `edit`; REJECTED stays `approve`.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="25">
       <c r="A100" s="27" t="inlineStr">
@@ -4792,15 +4839,19 @@
       </c>
       <c r="F100" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G100" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H100" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H100" s="48" t="inlineStr">
+        <is>
+          <t>doc/API_REFERENCE.md, GENERATED by scripts/generate-api-docs.js from doc/api-contract.json — the artefact check-api-contract.js already derives by mounting the real routers, and which CI already fails on. All 731 routes across 100 modules, grouped by prefix, with body-validation status. Critically it also documents THE OUT-OF-BAND REQUEST CONTRACT, which F-25 called out as underivable by an integrator: Host selects the tenant, X-Praxis-Env selects the sandbox schema for business data only, identity always resolves against LIVE so a TEST flip never logs you out, X-Request-Id correlation, and the list/filter/sort vocabulary. A generated spec cannot disagree with the code the way the 19%-complete Postman collection had. `--check` mode catches drift. NOT included: the access-tier table — see API-F23.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="34.5" customHeight="1" s="25">
       <c r="A101" s="27" t="inlineStr">
@@ -4914,15 +4965,19 @@
       </c>
       <c r="F103" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G103" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H103" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H103" s="48" t="inlineStr">
+        <is>
+          <t>FOUND BY TC-C12's chain test, not by inspection: asserting one error envelope across four failure modes showed the tenant-gate 404 had no request_id at all. hostTenantResolver (TENANT_NOT_FOUND / TENANT_SUSPENDED / TENANT_NOT_READY), tenantContext (NO_TENANT_CONTEXT) and feature-gate (NO_TENANT_CONTEXT / FEATURE_DISABLED) all answered with res.status(...).json(...) directly, bypassing the error handler — so the six failures a customer is most likely to phone about ('unknown workspace', 'workspace suspended', 'that feature is off') were the six they could not quote a correlation id for. Fixed STRUCTURALLY rather than by adding the field at six sites that would drift again: all six now go through next(new AppError(code, message, status)), so they inherit the standard envelope, the log line they never had, and — for the 500s — the error report. Status codes and error codes are unchanged, asserted explicitly. Verified: middleware-chain.test.js asserts request_id === the X-Request-Id header on all four gate failures and that the 404/403/423 contract is preserved; auth-middleware, rbac-enforcement and capability-assignment (62 assertions) re-run green.</t>
+        </is>
+      </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="25">
       <c r="A104" s="27" t="inlineStr">
@@ -4952,15 +5007,19 @@
       </c>
       <c r="F104" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G104" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H104" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H104" s="48" t="inlineStr">
+        <is>
+          <t>A tenant-API request on a platform host (localhost, api.*, admin.*, the apex) hit tenantContext with no req.tenant and answered 500 NO_TENANT_CONTEXT — a server error for a client mistake, and a documented footgun (postman/README warns 'localhost is the platform host'). tenantContext now distinguishes the two causes it was conflating: req.isPlatform means the resolver ran and deliberately set no tenant -&gt; 400 WRONG_HOST with a message naming the correct host and the X-Praxis-Tenant dev header. No tenant AND not a platform host still means a misordered middleware chain and stays a loud, logged, reported 500. Owner chose 400 over keeping the status.</t>
+        </is>
+      </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="25">
       <c r="A105" s="27" t="inlineStr">
@@ -5218,15 +5277,19 @@
       </c>
       <c r="F111" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G111" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H111" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H111" s="48" t="inlineStr">
+        <is>
+          <t>`update: create.partial()` made the status field patchable wherever create declared it, so PATCH /:id {status} reached a state change under plain `edit` while POST /:id/status might require `approve` — the transition gate was effectively optional, and tightening F-21 alone would have moved the hole rather than closed it. New shared middleware requireLifecyclePermissionOnPatch mounted on the PATCH route of all eleven affected resources: when the body does not carry the lifecycle field it does nothing at all, so ordinary edits are untouched; when it does, the request must satisfy the SAME permission the dedicated endpoint requires for that target state. A caller holding the right permission is unaffected; only the cheaper path 403s, which is the escalation closing. Owner chose enforce-now over shadow-mode.</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="25">
       <c r="A112" s="27" t="inlineStr">
@@ -5256,15 +5319,19 @@
       </c>
       <c r="F112" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G112" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H112" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H112" s="48" t="inlineStr">
+        <is>
+          <t>Two halves. (1) THE AUTHZ BUG: `react` and `star` took a bare messageId and asserted nothing, so any MOD-64 `view` holder could react to or star ANY message in ANY channel including ones they cannot see — and a reaction is broadcast over the realtime channel, so it doubled as a way to announce presence in a private conversation. `listMembers` likewise had no assert, disclosing any channel's roster. Added assertMessageMember (resolves message -&gt; channel, then the existing assertMember) and an assert on listMembers; the controller now passes the actor. Not-a-member and no-such-message return the SAME 403, so the message id is not disclosed. (2) THE CONTRACT: eight write endpoints were gated `view`, so granting a role MOD-64 view also granted 'add and remove channel members'. Writes to SHARED state (archive, add/remove member, edit/delete another's message) now require `edit`. Own-preference writes (pin, mute, read marker, draft, star, react) deliberately KEEP `view` and say so in writing — they are per-user rows keyed on the caller, and requiring a write grant to mute a channel you can already read would be the opposite mistake. Membership remains the real authorisation throughout.</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="25">
       <c r="A113" s="27" t="inlineStr">
@@ -5302,7 +5369,11 @@
           <t>As reported</t>
         </is>
       </c>
-      <c r="H113" s="28" t="n"/>
+      <c r="H113" s="48" t="inlineStr">
+        <is>
+          <t>ATTEMPTED AND DELIBERATELY NOT SHIPPED. The intent was to publish the self-scoped tier in the generated API reference. doc/api-contract.json records auth/rbac per route from the middleware NAMES on that route's own stack, but nearly every router applies authentication once via router.use(authMiddleware), which never appears on an individual route — so the flags read auth:false for hundreds of routes that ARE authenticated. Classifying tiers off them produced '713 public, 9 self-scoped' against the audit's 10 and 61. A security tier table that lies is worse than none, so the section was removed and replaced with an explicit statement of why, pointing at API_CONTRACT_AUDIT §F-23/F-24 as the reference meanwhile. Closing this properly means resolving router-level middleware inside check-api-contract.js so CI and the doc share one answer — a contained change, but it belongs to that script, not to a doc generator.</t>
+        </is>
+      </c>
     </row>
     <row r="114" ht="15" customHeight="1" s="25">
       <c r="A114" s="27" t="inlineStr">
@@ -5332,15 +5403,19 @@
       </c>
       <c r="F114" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G114" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H114" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H114" s="48" t="inlineStr">
+        <is>
+          <t>Unknown query keys were dropped silently, so `?stat=OPEN` returned the UNFILTERED list and looked like it had worked — a filter typo silently widened the result set. makeRepo now takes `filterable`; anything outside it (plus the shared limit/offset/q/sort vocabulary) is 422 UNKNOWN_FILTER naming the key and listing what is available. Declared on the 16 repos that use makeRepo's list unchanged — that list only ever honoured limit/offset/q, so every other key was already being ignored, which IS the finding. Repos that override list() keep current behaviour until their filters are declared, so nothing that works today breaks.</t>
+        </is>
+      </c>
     </row>
     <row r="115" ht="15" customHeight="1" s="25">
       <c r="A115" s="27" t="inlineStr">
@@ -5370,15 +5445,19 @@
       </c>
       <c r="F115" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G115" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H115" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H115" s="48" t="inlineStr">
+        <is>
+          <t>No endpoint accepted a sort parameter; order was fixed at makeRepo config time, so any consumer wanting a different order fetched and sorted client-side — and by F-26/F-27 that meant sorting a truncated 50-row window, i.e. sorting the wrong rows. `?sort=col` / `?sort=-col` now resolves through an explicit `sortable` allow-list (declared on all 24 makeRepo repos), validated and quoted via query-helpers.ident. An unlisted column is 422 INVALID_SORT listing what is sortable — refused, never interpolated, because ORDER BY built from user input is exactly the injection SEC H3 closed.</t>
+        </is>
+      </c>
     </row>
     <row r="116" ht="15" customHeight="1" s="25">
       <c r="A116" s="27" t="inlineStr">
@@ -5408,15 +5487,19 @@
       </c>
       <c r="F116" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G116" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H116" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H116" s="48" t="inlineStr">
+        <is>
+          <t>doc/ERROR_CODES.md, GENERATED from source by scripts/generate-api-docs.js: 219 AppError codes with raise counts and HTTP statuses, plus the shared error-envelope shape. The six near-synonyms the audit named (BAD_AMOUNT/INVALID_AMOUNT, BAD_STATE/BAD_STATUS, EMPLOYEE_NOT_FOUND/NOT_FOUND, FORBIDDEN + NOT_YOURS + NOT_A_MEMBER/PERMISSION_DENIED) are published as ALIASES, deliberately not renamed — a code a client already switches on cannot be changed without breaking it, and enumerating them is the precondition for ever retiring them. `--check` mode fails if the committed file drifts from the code.</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="15" customHeight="1" s="25">
       <c r="A117" s="27" t="inlineStr">
@@ -5728,15 +5811,19 @@
       </c>
       <c r="F124" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G124" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H124" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H124" s="28" t="inlineStr">
+        <is>
+          <t>New repo.preferencesFor / insertForUsers / activeEmailsFor and service.notifyMany. The fan-out called notify() per recipient, each issuing ~5 queries — for 50 finance users on invoice.posted (a normal path, it is on the allowlist) that is ~250 SEQUENTIAL round-trips while holding a write transaction open, pinning one of eight pooled connections and extending the lock window on the business row. Now a fixed 4 queries regardless of recipient count: one preference read for everyone across both channels, one multi-row INSERT via unnest (parameterised, so the statement text does not change with recipient count and the plan cache still works), one address lookup. MEASURED: 50 recipients went from ~250 round-trips to 2. Email/push sends deliberately stay in the caller's transaction — moving them out means deciding what happens when the transaction rolls back after an email has gone, which is a correctness question and a separate change.</t>
+        </is>
+      </c>
     </row>
     <row r="125" ht="15" customHeight="1" s="25">
       <c r="A125" s="27" t="inlineStr">
@@ -5766,15 +5853,19 @@
       </c>
       <c r="F125" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G125" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H125" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H125" s="28" t="inlineStr">
+        <is>
+          <t>emitEvent's first act on every create/update/archive across 93 modules was a SELECT on event_type — a STATIC SEEDED CATALOGUE, read on every single write and never cached. Now an in-process cache keyed by (tenant, key), because event_type is a tenant table and a global cache would let one tenant's catalogue answer another's question — the same mistake PERF S9 was about. 5-minute TTL so a process running since before a seeding migration notices within a deploy cycle; unknown keys cache as null too, since a nonexistent event type is a stable fact and not caching it leaves the hot path uncached for exactly the keys someone typo'd. Bounded at 5000 entries. MEASURED: 100 writes of the same event type went from 100 catalogue reads to 1, and a second tenant correctly missed.</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="15" customHeight="1" s="25">
       <c r="A126" s="27" t="inlineStr">
@@ -6090,15 +6181,19 @@
       </c>
       <c r="F133" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G133" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H133" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H133" s="48" t="inlineStr">
+        <is>
+          <t>auth-context.tsx passed an inline object literal as the provider value containing six handlers re-created on every render, so every render of AuthProvider produced a new context identity and re-rendered every consumer — and with zero React.memo across 134 components there was nothing to arrest the cascade. AuthProvider wraps the whole app, so that is every render of everything. All six handlers are now React.useCallback with empty deps (they close only over stable setters and module helpers; patchUser uses the functional setUser form, which is why it needs no user dep) and the value is useMemo'd, so its identity changes only when the auth state genuinely does. branding-context.tsx had the same shape and gets the same treatment. tsc --noEmit clean.</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="15" customHeight="1" s="25">
       <c r="A134" s="27" t="inlineStr">
@@ -6128,15 +6223,19 @@
       </c>
       <c r="F134" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G134" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H134" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H134" s="48" t="inlineStr">
+        <is>
+          <t>HALF OF THIS WAS ALREADY DONE and the register did not say so: client/src/lib/use-resource.ts is no longer the hand-rolled hook the audit describes — it has been migrated to TanStack Query (staleTime 30s, gcTime 5m, refetchOnWindowFocus), so caching, request dedup and stale-while-revalidate are in place across all 150+ call sites. What remained was the second half: app-shell.tsx's badge poller, a raw setInterval(load, 60000) OUTSIDE the cache, two requests per user per minute forever — the audit's arithmetic puts that at ~33 req/s of pure badge polling at 1,000 users and ~230 DB round-trips/second, on a topology with a 12-connection-per-tenant ceiling. Now a useQuery with refetchInterval 60s, refetchIntervalInBackground FALSE (most of that traffic was tabs nobody was looking at) and staleTime 30s, so the two requests are deduplicated across every component wanting a badge. refetchOnWindowFocus means returning to the tab refreshes immediately, so the badge is fresher on return while costing less in between. env is in the query key so a LIVE/TEST flip reads the right counts.</t>
+        </is>
+      </c>
     </row>
     <row r="135" ht="15" customHeight="1" s="25">
       <c r="A135" s="27" t="inlineStr">
@@ -6166,15 +6265,19 @@
       </c>
       <c r="F135" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G135" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H135" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H135" s="48" t="inlineStr">
+        <is>
+          <t>migrations/tenant/0504, part 2. pg_trgm GIN indexes on the 41 (table, column) pairs reachable by ILIKE — the 8 declared via makeRepo searchColumn plus 33 hand-rolled in module repos. A leading wildcard cannot use a B-tree, so every free-text search was a sequential scan; the audit measured 66.96ms -&gt; 4.55ms (14.7x) with no query rewrite, since the same SQL simply becomes indexable. The pair list was derived by static analysis and a `col ILIKE` inside a joining function cannot always be attributed to the right table from source alone, so rather than ship a list I could not fully verify — and fail the migration for every tenant on the first wrong pair — each index is created only if the column exists and is a text type, with a NOTICE naming any pair that does not resolve. That is explicitly NOT `EXCEPTION WHEN OTHERS THEN NULL` (DATA 3.6): the precondition is tested, and anything unexpected still aborts.</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="15" customHeight="1" s="25">
       <c r="A136" s="27" t="inlineStr">
@@ -6280,15 +6383,19 @@
       </c>
       <c r="F138" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G138" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H138" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H138" s="48" t="inlineStr">
+        <is>
+          <t>The identical hand-rolled `update()` SET builder was copy-pasted into 46 module repos. All 46 now call query-helpers.updateOne; zero remain (verified by grep). 39 were converted by a codemod that refuses anything it does not recognise exactly, and the 7 it reported were done by hand — including three genuinely different shapes (an arrow returning a promise chain, an object method using `this`, and one whose RETURNING is a module constant). updateOne gained an `opts.touch` option because appending `, updated_at = now()` was the sole reason most of them existed. Generated SQL verified byte-equivalent to the originals apart from identifier quoting.</t>
+        </is>
+      </c>
     </row>
     <row r="139" ht="15" customHeight="1" s="25">
       <c r="A139" s="27" t="inlineStr">
@@ -6318,15 +6425,19 @@
       </c>
       <c r="F139" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G139" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H139" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H139" s="48" t="inlineStr">
+        <is>
+          <t>The audit traced no live vulnerability and neither did I — but its point was that the helper should not depend on every caller being careful, and the real finding turned out to be sharper than 'defence in depth'. SEC H3 had already hardened query-helpers with identifier validation and an optional writable allow-list; what nobody had noticed is that the 46 repos in PERF-S19 BYPASSED IT ENTIRELY by building their own SET clause, so the hardening covered only the modules that happened to route through updateOne. Deduplicating those 46 is what makes it universal — S19 is the delivery mechanism for S20, not a separate tidy-up. Also fixed the one identifier still interpolated raw in that file: getById's `pk`. Verified: identifier injection now raises INVALID_FIELD and an out-of-list column raises FIELD_NOT_WRITABLE, on every repo.</t>
+        </is>
+      </c>
     </row>
     <row r="140" ht="15" customHeight="1" s="25">
       <c r="A140" s="27" t="inlineStr">
@@ -6650,15 +6761,19 @@
       </c>
       <c r="F147" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G147" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H147" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H147" s="28" t="inlineStr">
+        <is>
+          <t>tests/unit/money-path.test.js — 22 assertions running determination.compute FOR REAL against OHADA account codes: balance on every shape, VAT at 19.25% to the centime, receivable on the debit side of a sale (getting it backwards inverts the balance sheet and still balances), debours excluded from the taxable base (taxing it overstates output VAT to the revenue authority — a filing error, not just an invoice error), the purchase mirror, multi-line rounding where each line's VAT rounds independently, no zero-value legs, and all 9 refusal codes. Two of my own assertions were WRONG and the code was stricter than I assumed: toCents refuses sub-centime precision rather than rounding it, and refuses negative amounts rather than posting a contra. Both are better contracts than I expected and the tests now assert the real ones.</t>
+        </is>
+      </c>
     </row>
     <row r="148" ht="15" customHeight="1" s="25">
       <c r="A148" s="27" t="inlineStr">
@@ -6688,15 +6803,19 @@
       </c>
       <c r="F148" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G148" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H148" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H148" s="28" t="inlineStr">
+        <is>
+          <t>The four integration suites were never disabled by anyone — they self-skip on `!process.env.DATABASE_URL`, and nothing ever set it. journal-posting.test.js says so in its own header: 'Run in CI by adding a postgres service + db:provision, then set these vars.' The new migrations job is exactly that, so it now seeds a corporate_entity and the BQ/VT/AC/OD journals (not seeded by 9000-9060 — they are business data, not reference data) and runs the suites against the real database. The step asserts the PASS COUNT, not just the exit code, because Jest exits 0 on a run where every suite skipped — 'it passed' and 'it ran' are different questions and only one was ever being asked. mail-imap.test.js stays opt-in on live IMAP/SMTP credentials, which is correct: a test that talks to a third-party mail server does not belong in every PR run.</t>
+        </is>
+      </c>
     </row>
     <row r="149" ht="15" customHeight="1" s="25">
       <c r="A149" s="27" t="inlineStr">
@@ -6726,15 +6845,19 @@
       </c>
       <c r="F149" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G149" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H149" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H149" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/wms-inventory.test.js — 35 assertions on inventory.service and outbound.service. The three failures DATA 5.1 describes are concurrency and atomicity failures, so a canned fake would have passed against the BROKEN code just as happily as the fixed code (the objection TC-Q3 raises about the existing regex fakes). This file therefore does NOT mock the repo: it runs the real repo SQL against a small in-memory Postgres implementing per-row FOR UPDATE locks, delta-applied-to-stored-value semantics, the `qty_on_hand + $2 &gt;= 0` guard, and real BEGIN/COMMIT/ROLLBACK. That makes the actual failures testable: two concurrent -5 and -3 moves against 10 end at 2 (not 7 — the reported lost update) and genuinely serialise; two concurrent -6 against 10 let exactly ONE through and leave the balance at 4 with one journal row; twenty interleaved moves keep qty_on_hand equal to the sum of the journal and never negative; moves on DIFFERENT items do not serialise (row lock, not table lock); a failed move releases its lock. Also: the journal write failing rolls the balance back, the event write failing rolls both back, nested moves join one transaction rather than committing it early (DATA 5.2), and both state machines are asserted exhaustively as tables (14 stock transitions, 12 outbound). MUTATION-VERIFIED: restoring the pre-DATA-5.1 read-modify-write move() fails 9 of the 35, including both race tests. Two fixture defects were found and fixed while writing this — a rollback that truncated the journal to a high-water mark (which rolled back a CONCURRENT transaction's committed work) and a non-re-entrant row lock that self-deadlocked nested moves; both are commented in place.</t>
+        </is>
+      </c>
     </row>
     <row r="150" ht="15" customHeight="1" s="25">
       <c r="A150" s="27" t="inlineStr">
@@ -6764,15 +6887,19 @@
       </c>
       <c r="F150" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G150" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H150" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H150" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/orchestration-outbox.test.js — all 10 assertions now pass end to end (previously 7-8 then an undiagnosed hang, which is why this was left Partially fixed). THE HANG WAS NOT A HANG. `jest.resetModules()` in beforeEach made every one of the ten tests rebuild the dispatcher's require graph, which is 171 modules because dispatcher.js requires ./handlers at load. Measured: ~6s per rebuild on a mounted filesystem, ~8.3s cold — ten tests is ~60s, so the file died around test seven or eight with no failure and no summary. Diagnosed by requiring the dispatcher in a bare node process: it leaves ZERO active handles beyond stdio and the process exits cleanly, so there is no leaked timer or connection — the previous session's stated suspicion was the wrong premise. The reset is also unnecessary: the dispatcher holds no module-level mutable state (every sweep's state is on the client the caller passes) and resolves handlers through registry.getHandlers() at dispatch time, so the mock picks up each test's handler list with nothing reloaded. Fix: require the dispatcher once at file load, keep only `handlers = []` in beforeEach. Runtime 60s+ -&gt; 8.5s. The jest.setup.js ALERT_WEBHOOK_URL/ALERT_EMAIL fix from the previous session stands and is unrelated.</t>
+        </is>
+      </c>
     </row>
     <row r="151" ht="15" customHeight="1" s="25">
       <c r="A151" s="27" t="inlineStr">
@@ -6802,15 +6929,19 @@
       </c>
       <c r="F151" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G151" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H151" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H151" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/tenant-provisioning.test.js — 52 assertions on provisioning.service, the code scripts/deploy.sh runs against every tenant on every deploy. Concentrated on the three behaviours that are themselves fixes for other findings and had no coverage: (1) DATA 3.2 fleet containment — a failing tenant no longer aborts the sweep, asserted by failing the MIDDLE of three and proving the third was still migrated, that each tenant is enumerated with which side of the line it fell on, and that it still throws FLEET_MIGRATION_PARTIAL afterwards so a deploy goes red; (2) the citext[] depends_on trap — toDepsArray parses the raw Postgres literal ('{}' -&gt; [], never ['{','}']), enforceDependencies cascades to a fixpoint through a chain and in any row order, an unknown dependency counts as unmet, source is preserved while state flips, and the query still carries the ::text[] cast; (3) SEC H6 on createAdmin, which mints the CEO account that bypasses every permission check. Also: slug rejection (it becomes a database name), unknown plan refused before the tenant goes LIVE, provisioning order, both schemas migrated, secret_ref is a pointer not a password, wipeSandbox clearing ONLY the sandbox migration scopes, and fleetSchemaStatus reporting an unreachable tenant rather than failing the report. MUTATION-VERIFIED: five simultaneous mutations (abort-on-first-failure, dropped ::text[] cast, single-pass fixpoint, removed SEC H6 check, full ledger wipe) fail 11 of the 52. Two honest notes: a dependency CYCLE is left on rather than off — recorded in the test, unreachable from the current catalogue, not claimed as a finding; and wipeSandbox's non-transactionality (DI-5.6, still Open) is asserted as current behaviour so whoever fixes it sees the test fail deliberately.</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="15" customHeight="1" s="25">
       <c r="A152" s="27" t="inlineStr">
@@ -6840,15 +6971,19 @@
       </c>
       <c r="F152" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G152" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H152" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H152" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/portal-auth.test.js — 45 assertions across portal_auth.service AND portal_auth.middleware, which is where the grant is actually enforced. Four properties: (1) a portal token is not a staff token — both are signed with JWT_ACCESS_SECRET so typ is the entire boundary, asserted from both directions (staff access token, 2FA-pending token and refresh-secret-signed token all refused, at the service AND at the gate); (2) the token carries identity only and portal_access is re-read per request, asserted by pulling the grant between two calls with the SAME token and getting 403; (3) failures do not enumerate — unknown email / wrong password / disabled account produce one error, and unknown / used / expired / empty invite tokens produce one error, asserted by comparing the errors to EACH OTHER rather than to a string literal; (4) SEC H6 holds — 'password' and '12345678', the two that passed the old `length &lt; 8` check, are named explicitly. Also covers invite lifetimes (7 days vs 30 minutes, 0482), one-live-link-at-a-time, tokens stored hashed, a weak password NOT consuming the invite, mail failure preserving both the login and the token, and a disabled account being re-activated on re-invite. argon2, jwt and the password policy are real; only the repo, mailer and portal-access lookup are mocked. MUTATION-VERIFIED: removing the typ check, the SEC H6 policy call, the grant check and the ACTIVE-status check fails 10 of the 45.</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="15" customHeight="1" s="25">
       <c r="A153" s="27" t="inlineStr">
@@ -6878,15 +7013,19 @@
       </c>
       <c r="F153" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G153" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H153" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H153" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/middleware-chain.test.js — 42 assertions sending real HTTP through supertest into a real Express app with the real chain (requestId -&gt; hostTenantResolver -&gt; tenantContext -&gt; authMiddleware -&gt; requirePermission -&gt; controller). Express, the router, the async-safe shim and all five middlewares are real; only the tenant registry and identity cache are mocked. Asserts what only a chain can: ORDER (tenantContext without the resolver, and auth without tenantContext, both 500 rather than proceeding tenant-less, and the identity cache is never reached); SHORT-CIRCUIT (a SUSPENDED tenant is 403 and a PROVISIONING tenant 423 even when a perfectly valid token is presented — asserted WITH a valid token, and getAuthUser is never called); PERF S2 (exactly ONE connection checkout for a request where auth, rbac and the controller all read — the fix was for three, capping concurrency at pool_max/3 — plus zero checkouts for a route that touches no database, and a search_path re-bind rather than a second checkout under sandbox); OBS-E3 (the correlation id from header to ambient context to error body, client-supplied ids adopted, over-long ones rejected); OBS-L3 (auth back-filling userId into the context tenantContext bound before it); SEC-C2 sid; the LIVE/TEST toggle not logging the user out; CEO bypass; and `=== true` grant comparison rejecting a truthy 1. Two hosts resolve to two tenants in one process.</t>
+        </is>
+      </c>
     </row>
     <row r="154" ht="15" customHeight="1" s="25">
       <c r="A154" s="27" t="inlineStr">
@@ -6916,15 +7055,19 @@
       </c>
       <c r="F154" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G154" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H154" s="28" t="n"/>
+          <t>Verified in code</t>
+        </is>
+      </c>
+      <c r="H154" s="48" t="inlineStr">
+        <is>
+          <t>tests/unit/auth-refresh-flow.test.js — 22 assertions on refresh() ITSELF, not on its extracted predicate. The audit's objection was that a refactor dropping the refreshTokenReused call site would leave all five existing predicate tests passing; PROVEN BY MUTATION: disabling that call site fails 3 of the new tests and 0 of the 5 old ones. Covers typ-confusion (an access token presented as a refresh token), wrong-secret rejection, expiry, killed session, subject/session mismatch, reuse-of-a-rotated-away-token asserted END TO END (rotate once, replay the original — no reference to the predicate by name), that revocation is complete (row killed + Redis removed + identity cache invalidated + LOGGED_OUT with reason refresh_token_reuse), that a revoked session is not simultaneously rotated or touched, legacy NULL-jti grandfathering, the 30-min inactivity kill and its exact boundary (the check is &gt; not &gt;=), keep_signed_in opting out of the idle kill but NOT out of revocation (0494), NaN-safe idle handling, and sid surviving rotation (SEC-C2). Two further mutations verified: dropping sid from the rotated access token and widening the idle window each fail exactly the test that names them. JWT is real throughout — tokens are signed and verified with the configured secrets.</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="15" customHeight="1" s="25">
       <c r="A155" s="27" t="inlineStr">
@@ -6954,15 +7097,19 @@
       </c>
       <c r="F155" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G155" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H155" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H155" s="28" t="inlineStr">
+        <is>
+          <t>Same file. final-invoice-lifecycle.test.js mocks determination and journal_entry.service, so it asserts the lifecycle and NOTHING about the accounting — which is correct for a lifecycle test; the missing half was a test of the arithmetic itself. That half now exists and is unmocked. The balance assertion is the load-bearing one: assert_entry_balanced in the database is the final authority but fires at INSERT time, by which point the failure surfaces as a 500 from inside a posting.</t>
+        </is>
+      </c>
     </row>
     <row r="156" ht="15" customHeight="1" s="25">
       <c r="A156" s="27" t="inlineStr">
@@ -6992,15 +7139,19 @@
       </c>
       <c r="F156" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G156" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H156" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H156" s="28" t="inlineStr">
+        <is>
+          <t>New `migrations` job: postgres:16 service, real platform migrate, a tenant provisioned from nothing (the path a new customer takes, never previously run in CI), then the tenant set applied a SECOND time asserting zero files applied — the migrator's idempotency claim rests entirely on its schema_migration ledger and nothing checked it. Then probe-doc-numbers, because 0498's unique indexes have no NOT VALID escape and either build or fail the whole run. This is the worst asymmetry in the audit: every other gate's worst outcome is a broken feature; a migration's is a half-migrated production database at the moment deploy.sh has already rolled the old image away.</t>
+        </is>
+      </c>
     </row>
     <row r="157" ht="15" customHeight="1" s="25">
       <c r="A157" s="27" t="inlineStr">
@@ -7030,15 +7181,19 @@
       </c>
       <c r="F157" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G157" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H157" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H157" s="28" t="inlineStr">
+        <is>
+          <t>docker-build now STARTS the image and waits for /api/health, then asserts every module mounts inside it. The image was built and never run, so anything between `docker build` succeeding and the process serving reached production untouched — which is not hypothetical: the deps stage did not copy packages/, so the image shipped with @praxis/shared unresolvable and NO INVOICING MODULE, and it built perfectly. Liveness only, because /api/health deliberately touches no dependency and is the one question a container with no database can answer. Runs with NODE_ENV=production — verified the throwaway CI secrets satisfy env.js's production guard, which rejects the dev-default ENCRYPTION_KEY and identical access/refresh secrets.</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="15" customHeight="1" s="25">
       <c r="A158" s="27" t="inlineStr">
@@ -7068,15 +7223,19 @@
       </c>
       <c r="F158" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G158" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H158" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H158" s="28" t="inlineStr">
+        <is>
+          <t>npm ci everywhere (4 sites). The old comment justified `install` on the grounds that the lockfile is Windows-generated so `ci` could omit linux binaries — THE PREMISE IS FALSE and was worth checking rather than inheriting: lockfileVersion 3 records every platform variant regardless of the generating machine, verified that this lockfile contains @img/sharp-linux-x64, @img/sharp-libvips-linux-x64, argon2 and node-gyp-build. The cost of the old line is the finding: `npm install` may resolve NEWER versions than the lockfile pins, so CI tested a dependency tree that is neither what the Dockerfile builds nor what deploys.</t>
+        </is>
+      </c>
     </row>
     <row r="159" ht="15" customHeight="1" s="25">
       <c r="A159" s="27" t="inlineStr">
@@ -7106,15 +7265,19 @@
       </c>
       <c r="F159" s="28" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="G159" s="28" t="inlineStr">
         <is>
-          <t>As reported</t>
-        </is>
-      </c>
-      <c r="H159" s="28" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="H159" s="28" t="inlineStr">
+        <is>
+          <t>Same fix as DI-3.2 — this finding IS the containment half. Per-tenant error capture, an enumerated result, a FLEET_MIGRATION_PARTIAL error carrying the full outcome, and a read-only status command that names who is behind and who is unreachable (which are different problems: unreachable is not behind, and migrating an unreachable tenant is not the remedy).</t>
+        </is>
+      </c>
     </row>
     <row r="160" ht="15" customHeight="1" s="25">
       <c r="A160" s="27" t="inlineStr">
@@ -9410,27 +9573,27 @@
         </is>
       </c>
       <c r="B5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G5" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A5,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A5,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H5" s="46">
@@ -9445,27 +9608,27 @@
         </is>
       </c>
       <c r="B6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G6" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A6,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A6,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H6" s="46">
@@ -9480,27 +9643,27 @@
         </is>
       </c>
       <c r="B7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G7" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A7,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A7,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H7" s="46">
@@ -9515,27 +9678,27 @@
         </is>
       </c>
       <c r="B8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G8" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A8,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A8,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H8" s="46">
@@ -9550,27 +9713,27 @@
         </is>
       </c>
       <c r="B9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G9" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A9,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A9,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H9" s="46">
@@ -9585,27 +9748,27 @@
         </is>
       </c>
       <c r="B10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G10" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A10,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A10,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H10" s="46">
@@ -9620,27 +9783,27 @@
         </is>
       </c>
       <c r="B11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,B$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,B$4)</f>
         <v/>
       </c>
       <c r="C11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,C$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,C$4)</f>
         <v/>
       </c>
       <c r="D11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,D$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,D$4)</f>
         <v/>
       </c>
       <c r="E11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,E$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,E$4)</f>
         <v/>
       </c>
       <c r="F11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,F$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,F$4)</f>
         <v/>
       </c>
       <c r="G11" s="46">
-        <f>COUNTIFS(Register!$B$2:$B$206,$A11,Register!$D$2:$D$206,G$4)</f>
+        <f>COUNTIFS(Register!$B$2:$B$500,$A11,Register!$D$2:$D$500,G$4)</f>
         <v/>
       </c>
       <c r="H11" s="46">
@@ -9714,7 +9877,7 @@
         </is>
       </c>
       <c r="B15" s="46">
-        <f>COUNTIF(Register!$F$2:$F$206,$A15)</f>
+        <f>COUNTIF(Register!$F$2:$F$500,$A15)</f>
         <v/>
       </c>
       <c r="C15" s="46" t="n"/>
@@ -9731,7 +9894,7 @@
         </is>
       </c>
       <c r="B16" s="46">
-        <f>COUNTIF(Register!$F$2:$F$206,$A16)</f>
+        <f>COUNTIF(Register!$F$2:$F$500,$A16)</f>
         <v/>
       </c>
       <c r="C16" s="46" t="n"/>
@@ -9748,7 +9911,7 @@
         </is>
       </c>
       <c r="B17" s="46">
-        <f>COUNTIF(Register!$F$2:$F$206,"Fixed")</f>
+        <f>COUNTIF(Register!$F$2:$F$500,"Fixed")</f>
         <v/>
       </c>
       <c r="C17" s="46" t="n"/>
@@ -9765,7 +9928,7 @@
         </is>
       </c>
       <c r="B18" s="46">
-        <f>COUNTIF(Register!$F$2:$F$206,$A18)</f>
+        <f>COUNTIF(Register!$F$2:$F$500,$A18)</f>
         <v/>
       </c>
       <c r="C18" s="46" t="n"/>
@@ -9782,7 +9945,7 @@
         </is>
       </c>
       <c r="B19" s="46">
-        <f>COUNTIF(Register!$F$2:$F$206,$A19)</f>
+        <f>COUNTIF(Register!$F$2:$F$500,$A19)</f>
         <v/>
       </c>
       <c r="C19" s="46" t="n"/>
@@ -9799,7 +9962,7 @@
         </is>
       </c>
       <c r="B20" s="46">
-        <f>COUNTIF(Register!$G$2:$G$206,"Verified in code")</f>
+        <f>COUNTIF(Register!$G$2:$G$500,"Verified in code")</f>
         <v/>
       </c>
       <c r="C20" s="46" t="n"/>

</xml_diff>